<commit_message>
trc khi sửa log
</commit_message>
<xml_diff>
--- a/codedoan4/data/input_case.xlsx
+++ b/codedoan4/data/input_case.xlsx
@@ -3,8 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Dangnhap" sheetId="1" r:id="rId1"/>
-    <sheet name="Dangky" sheetId="2" r:id="rId2"/>
+    <sheet name="Dangky" sheetId="1" r:id="rId1"/>
+    <sheet name="Dangnhap" sheetId="2" r:id="rId2"/>
     <sheet name="Hsotkhoan" sheetId="3" r:id="rId3"/>
     <sheet name="Timkiem" sheetId="4" r:id="rId4"/>
     <sheet name="Muahang" sheetId="5" r:id="rId5"/>
@@ -401,205 +401,357 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:G24"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
+        <v>tentaikhoan</v>
+      </c>
+      <c r="B1" t="str">
         <v>email</v>
       </c>
-      <c r="B1" t="str">
+      <c r="C1" t="str">
         <v>matkhau</v>
       </c>
-      <c r="C1" t="str">
+      <c r="D1" t="str">
         <v>ketquamongdoi</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>hoangnguyet@gmail.com</v>
+        <v/>
       </c>
       <c r="B2" t="str">
-        <v>1423Nguyet*</v>
+        <v>thu2h312oangTthuyduye12345671nn@gmail.com</v>
       </c>
       <c r="C2" t="str">
-        <v>Lỗi: Mật khẩu bạn nhập cho địa chỉ email hoangnguyet@gmail.com không đúng. Bạn quên mật khẩu?</v>
+        <v/>
+      </c>
+      <c r="D2" t="str">
+        <v>Xin chào thu2h312oangtthuyduye12345671nn (không phải thu2h312oangtthuyduye12345671nn? Đăng xuất)</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>HoangMinhNguyet110122277@gmail.com</v>
+        <v>thúy duyên</v>
       </c>
       <c r="B3" t="str">
-        <v>1424Nguyet*</v>
+        <v>hoangthuyduyen311@gmail.com</v>
       </c>
       <c r="C3" t="str">
-        <v>Xin chào Minh Nguyệt (không phải Minh Nguyệt? Đăng xuất)</v>
+        <v/>
+      </c>
+      <c r="D3" t="str">
+        <v>Đã có tài khoản đăng ký với tên đăng nhập này. Vui lòng chọn tên khác.</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>duyen123@gmail.com</v>
+        <v/>
       </c>
       <c r="B4" t="str">
-        <v>1424Nguyet*</v>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="C4" t="str">
-        <v>Địa chỉ email không xác định. Kiểm tra lại hoặc thử tên người dùng của bạn.</v>
+        <v>thuyduyen22</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Lỗi: Vui lòng cung cấp địa chỉ email hợp lệ.</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v/>
+        <v>thúy duyên</v>
       </c>
       <c r="B5" t="str">
-        <v>1424Nguyet*</v>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="C5" t="str">
-        <v>Lỗi: Yêu cầu tên tài khoản.</v>
+        <v/>
+      </c>
+      <c r="D5" t="str">
+        <v>Lỗi: Vui lòng cung cấp địa chỉ email hợp lệ.</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>hoangnguyet@gmail.com</v>
+        <v/>
       </c>
       <c r="B6" t="str">
-        <v/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="C6" t="str">
-        <v>Lỗi: Trường mật khẩu đang trống.</v>
+        <v/>
+      </c>
+      <c r="D6" t="str">
+        <v>Lỗi: Vui lòng cung cấp địa chỉ email hợp lệ.</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v/>
+        <v>12345</v>
       </c>
       <c r="B7" t="str">
-        <v/>
+        <v>hoangnguyet@gmail.com</v>
       </c>
       <c r="C7" t="str">
-        <v>Lỗi: Yêu cầu tên tài khoản.</v>
+        <v/>
+      </c>
+      <c r="D7" t="str">
+        <v>Lỗi: Một tài khoản đã được đăng ký với hoangnguyet@gmail.com. Vui lòng đăng nhập hoặc sử dụng địa chỉ email khác.</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>hoangnguyetgmail.com</v>
+        <v>ban@!</v>
       </c>
       <c r="B8" t="str">
-        <v>1424Nguyet*</v>
+        <v>hoanghang@gmai.com</v>
       </c>
       <c r="C8" t="str">
-        <v>Lỗi: Tên người dùng hoangnguyetgmail.com không được đăng ký trên trang web này. Nếu bạn không chắc về tên người dùng của mình, hãy thử địa chỉ email của bạn.</v>
+        <v/>
+      </c>
+      <c r="D8" t="str">
+        <v>Lỗi: Tên tài khoản không được gồm ký tự Đặc biệt.</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>hoangduyen@gmail.com</v>
+        <v>tienbao1</v>
       </c>
       <c r="B9" t="str">
-        <v>duyen</v>
+        <v>thu1baohoang1@gmail.com</v>
       </c>
       <c r="C9" t="str">
-        <v>Địa chỉ email không xác định. Kiểm tra lại hoặc thử tên người dùng của bạn.</v>
+        <v>abc</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Độ mạnh mật khẩu: Rất yếu - Vui lòng nhập mật khẩu mạnh hơn.</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>hoangnguyet@gmai.com</v>
+        <v>tienbao</v>
       </c>
       <c r="B10" t="str">
-        <v>1424Nguyet*</v>
+        <v>baohoang11@gmail.com</v>
       </c>
       <c r="C10" t="str">
-        <v>Địa chỉ email không xác định. Kiểm tra lại hoặc thử tên người dùng của bạn.</v>
+        <v>abc12345</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Độ mạnh mật khẩu: Yếu - Vui lòng nhập mật khẩu mạnh hơn.</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>hoangnguyet@gmai.com</v>
+        <v>@##@$%</v>
       </c>
       <c r="B11" t="str">
-        <v>Nguyet1424*</v>
+        <v>hoanghang@gmai.com</v>
       </c>
       <c r="C11" t="str">
-        <v>Địa chỉ email không xác định. Kiểm tra lại hoặc thử tên người dùng của bạn.</v>
+        <v/>
+      </c>
+      <c r="D11" t="str">
+        <v>Lỗi: Tên tài khoản không được gồm ký tự Đặc biệt.</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>hoangnguyet$$gmail.com</v>
+        <v>thúy duyên</v>
       </c>
       <c r="B12" t="str">
-        <v>1424Nguyet*</v>
+        <v>hoangthuyduyen311</v>
       </c>
       <c r="C12" t="str">
-        <v>Lỗi: Tên người dùng hoangnguyet$$gmail.com không được đăng ký trên trang web này. Nếu bạn không chắc về tên người dùng của mình, hãy thử địa chỉ email của bạn.</v>
+        <v>thuyduyen22</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Please include an '@' in the email address. 'hoangthuyduyen311' is missing an '@'.</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>thúy duyên</v>
+      </c>
+      <c r="B13" t="str">
+        <v>hoangthuyduyen311@@gmail.com</v>
+      </c>
+      <c r="C13" t="str">
+        <v>thuyduyen22</v>
+      </c>
+      <c r="D13" t="str">
+        <v>A part following '@' should not contain the symbol '@'.</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>thúy duyên</v>
+      </c>
+      <c r="B14" t="str">
+        <v>hoangthuyduyen311gmail.com</v>
+      </c>
+      <c r="C14" t="str">
+        <v>thuyduyen22</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Please include an '@' in the email address. 'hoangthuyduyen311gmail.com' is missing an '@'.</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>thúy duyên</v>
+      </c>
+      <c r="B15" t="str">
+        <v>@gmai.comm</v>
+      </c>
+      <c r="C15" t="str">
+        <v>thuyduyen22</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Please enter a part followed by '@'. '@gmai.comm' is incomplete.</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>vân1</v>
+      </c>
+      <c r="B16" t="str">
+        <v>vannguyen@gmail.com31</v>
+      </c>
+      <c r="C16" t="str">
+        <v>thuyduyen22</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Xin chào van1 (không phải van1? Đăng xuất)</v>
+      </c>
+      <c r="G16" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>t2</v>
+      </c>
+      <c r="B17" t="str">
+        <v>thudoanl1@gmail.com</v>
+      </c>
+      <c r="C17" t="str">
+        <v>minhnguyet1@</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Xin chào t2 (không phải t2? Đăng xuất)</v>
+      </c>
+      <c r="E17" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v xml:space="preserve">NguyễnHoàngĐìnhVũTrấnLiênBỉnhPhátAnhQuânHoàngNguyênTuấnTàiBảoNamDuyênDungTiênDươngHườngThếNgânNamDũngLợiNgọcHiềnTrungHươngThìnHòaBìnhNguyễnHoàngĐìnhVũAnhQuânBỉnhPhátNguyênTuấnBảoNamDuyênDungTiênDươngHườngThếNgânDũngLợiNgọcHiềnTrungHươngThìnHòaBình </v>
+      </c>
+      <c r="B18" t="str">
+        <v>thudoanl21@gmail.com</v>
+      </c>
+      <c r="C18" t="str">
+        <v>minhnguyet1</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Lỗi: Tên người dùng không thể dài hơn 60 kí tự.</v>
+      </c>
+      <c r="G18" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>duyn1</v>
+      </c>
+      <c r="B19" t="str">
+        <v>thudoanl21 @gmail.com</v>
+      </c>
+      <c r="C19" t="str">
+        <v>minhnguyet1</v>
+      </c>
+      <c r="D19" t="str">
+        <v>A part followed by '@' should not contain the symbol ' '.</v>
+      </c>
+      <c r="E19" t="str">
+        <v/>
+      </c>
+      <c r="G19" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="G20" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="G21" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="G24" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G24"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:C11"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>tentaikhoan</v>
+        <v>email</v>
       </c>
       <c r="B1" t="str">
-        <v>email</v>
+        <v>matkhau</v>
       </c>
       <c r="C1" t="str">
-        <v>matkhau</v>
-      </c>
-      <c r="D1" t="str">
         <v>ketquamongdoi</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>thúy duyên</v>
+        <v>hoangnguyet@gmail.com</v>
       </c>
       <c r="B2" t="str">
-        <v>hoangthuyduyen311@gmail.com</v>
+        <v>1423Nguyet*</v>
       </c>
       <c r="C2" t="str">
-        <v/>
-      </c>
-      <c r="D2" t="str">
-        <v>Đã có tài khoản đăng ký với tên đăng nhập này. Vui lòng chọn tên khác.</v>
+        <v>Lỗi: Mật khẩu bạn nhập cho địa chỉ email hoangnguyet@gmail.com không đúng. Bạn quên mật khẩu?</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v/>
+        <v>HoangMinhNguyet110122277@gmail.com</v>
       </c>
       <c r="B3" t="str">
-        <v xml:space="preserve"> </v>
+        <v>1424Nguyet*</v>
       </c>
       <c r="C3" t="str">
-        <v>thuyduyen22</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Lỗi: Vui lòng cung cấp địa chỉ email hợp lệ.</v>
+        <v>Xin chào Minh Nguyệt (không phải Minh Nguyệt? Đăng xuất)</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>thúy duyên</v>
+        <v>duyen123@gmail.com</v>
       </c>
       <c r="B4" t="str">
-        <v xml:space="preserve"> </v>
+        <v>1424Nguyet*</v>
       </c>
       <c r="C4" t="str">
-        <v/>
-      </c>
-      <c r="D4" t="str">
-        <v>Lỗi: Vui lòng cung cấp địa chỉ email hợp lệ.</v>
+        <v>Địa chỉ email không xác định. Kiểm tra lại hoặc thử tên người dùng của bạn.</v>
       </c>
     </row>
     <row r="5">
@@ -607,223 +759,88 @@
         <v/>
       </c>
       <c r="B5" t="str">
-        <v xml:space="preserve"> </v>
+        <v>1424Nguyet*</v>
       </c>
       <c r="C5" t="str">
-        <v/>
-      </c>
-      <c r="D5" t="str">
-        <v>Lỗi: Vui lòng cung cấp địa chỉ email hợp lệ.</v>
+        <v>Lỗi: Yêu cầu tên tài khoản.</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v/>
+        <v>hoangnguyet@gmail.com</v>
       </c>
       <c r="B6" t="str">
-        <v>h312oangTthuyduye12345671nn@gmail.com</v>
+        <v/>
       </c>
       <c r="C6" t="str">
-        <v/>
-      </c>
-      <c r="D6" t="str">
-        <v>Xin chào h312oangtthuyduye12345671nn (không phải h312oangtthuyduye12345671nn? Đăng xuất)</v>
+        <v>Lỗi: Trường mật khẩu đang trống.</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>12345</v>
+        <v/>
       </c>
       <c r="B7" t="str">
-        <v>hoangnguyet@gmail.com</v>
+        <v/>
       </c>
       <c r="C7" t="str">
-        <v/>
-      </c>
-      <c r="D7" t="str">
-        <v>Lỗi: Một tài khoản đã được đăng ký với hoangnguyet@gmail.com. Vui lòng đăng nhập hoặc sử dụng địa chỉ email khác.</v>
+        <v>Lỗi: Yêu cầu tên tài khoản.</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>ban@!</v>
+        <v>hoangnguyetgmail.com</v>
       </c>
       <c r="B8" t="str">
-        <v>hoanghang@gmai.com</v>
+        <v>1424Nguyet*</v>
       </c>
       <c r="C8" t="str">
-        <v/>
-      </c>
-      <c r="D8" t="str">
-        <v>Lỗi: Tên tài khoản không được gồm ký tự Đặc biệt.</v>
+        <v>Lỗi: Tên người dùng hoangnguyetgmail.com không được đăng ký trên trang web này. Nếu bạn không chắc về tên người dùng của mình, hãy thử địa chỉ email của bạn.</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>tienbao</v>
+        <v xml:space="preserve">    hoangnguyet@gmai.com</v>
       </c>
       <c r="B9" t="str">
-        <v>baohoang1@gmail.com</v>
+        <v>1424 Nguyet*</v>
       </c>
       <c r="C9" t="str">
-        <v>abc</v>
-      </c>
-      <c r="D9" t="str">
-        <v>Độ mạnh mật khẩu: Rất yếu - Vui lòng nhập mật khẩu mạnh hơn.</v>
+        <v>Địa chỉ email không xác định. Kiểm tra lại hoặc thử tên người dùng của bạn.</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>tienbao</v>
+        <v>hoangnguyet@gmai.com</v>
       </c>
       <c r="B10" t="str">
-        <v>baohoang11@gmail.com</v>
+        <v xml:space="preserve">   Nguyet1424*</v>
       </c>
       <c r="C10" t="str">
-        <v>abc12345</v>
-      </c>
-      <c r="D10" t="str">
-        <v>Độ mạnh mật khẩu: Yếu - Vui lòng nhập mật khẩu mạnh hơn.</v>
+        <v>Địa chỉ email không xác định. Kiểm tra lại hoặc thử tên người dùng của bạn.</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>@##@$%</v>
+        <v>hoangnguyet$$gmail.com</v>
       </c>
       <c r="B11" t="str">
-        <v>hoanghang@gmai.com</v>
+        <v>1424Nguyet*</v>
       </c>
       <c r="C11" t="str">
-        <v/>
-      </c>
-      <c r="D11" t="str">
-        <v>Lỗi: Tên tài khoản không được gồm ký tự Đặc biệt.</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>thúy duyên</v>
-      </c>
-      <c r="B12" t="str">
-        <v>hoangthuyduyen311</v>
-      </c>
-      <c r="C12" t="str">
-        <v>thuyduyen22</v>
-      </c>
-      <c r="D12" t="str">
-        <v>Please include an '@' in the email address. 'hoangthuyduyen311' is missing an '@'.</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>thúy duyên</v>
-      </c>
-      <c r="B13" t="str">
-        <v>hoangthuyduyen311@@gmail.com</v>
-      </c>
-      <c r="C13" t="str">
-        <v>thuyduyen22</v>
-      </c>
-      <c r="D13" t="str">
-        <v>A part following '@' should not contain the symbol '@'.</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>thúy duyên</v>
-      </c>
-      <c r="B14" t="str">
-        <v>hoangthuyduyen311gmail.com</v>
-      </c>
-      <c r="C14" t="str">
-        <v>thuyduyen22</v>
-      </c>
-      <c r="D14" t="str">
-        <v>Please include an '@' in the email address. 'hoangthuyduyen311gmail.com' is missing an '@'.</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>thúy duyên</v>
-      </c>
-      <c r="B15" t="str">
-        <v>@gmai.comm</v>
-      </c>
-      <c r="C15" t="str">
-        <v>thuyduyen22</v>
-      </c>
-      <c r="D15" t="str">
-        <v>Please enter a part followed by '@'. '@gmai.comm' is incomplete.</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="str">
-        <v>vân</v>
-      </c>
-      <c r="B16" t="str">
-        <v>vannguyen@gmail.com31</v>
-      </c>
-      <c r="C16" t="str">
-        <v>thuyduyen22</v>
-      </c>
-      <c r="D16" t="str">
-        <v>Xin chào van (không phải van? Đăng xuất)</v>
-      </c>
-      <c r="G16" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="E17" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="G18" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="E19" t="str">
-        <v/>
-      </c>
-      <c r="G19" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="E20" t="str">
-        <v/>
-      </c>
-      <c r="G20" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="G21" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="G22" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="25">
-      <c r="G25" t="str">
-        <v/>
+        <v>Lỗi: Tên người dùng hoangnguyet$$gmail.com không được đăng ký trên trang web này. Nếu bạn không chắc về tên người dùng của mình, hãy thử địa chỉ email của bạn.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G25"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C11"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J22"/>
+  <dimension ref="A1:J27"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1299,9 +1316,9 @@
         <v/>
       </c>
       <c r="J15" t="str" xml:space="preserve">
-        <v xml:space="preserve">Tên là mục bắt buộc._x000d_
-Họ là mục bắt buộc._x000d_
-Tên hiển thị là mục bắt buộc._x000d_
+        <v xml:space="preserve">Tên là mục bắt buộc._x000d__x000d__x000d__x000d_
+Họ là mục bắt buộc._x000d__x000d__x000d__x000d_
+Tên hiển thị là mục bắt buộc._x000d__x000d__x000d__x000d_
 Địa chỉ email là mục bắt buộc.</v>
       </c>
     </row>
@@ -1502,9 +1519,138 @@
         <v>Thông tin tài khoản đã được cập nhật.</v>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>dung@gmail.com</v>
+      </c>
+      <c r="B23" t="str">
+        <v>dungtoan1</v>
+      </c>
+      <c r="C23" t="str">
+        <v>dung</v>
+      </c>
+      <c r="D23" t="str">
+        <v>nguyen</v>
+      </c>
+      <c r="E23" t="str">
+        <v>DUNG</v>
+      </c>
+      <c r="F23" t="str">
+        <v>dung@GMAIL.COM</v>
+      </c>
+      <c r="J23" t="str">
+        <v>Địa chỉ email này đã được đăng ký và sử dụng.</v>
+      </c>
+    </row>
+    <row r="24" xml:space="preserve">
+      <c r="A24" t="str">
+        <v>dung@gmail.com</v>
+      </c>
+      <c r="B24" t="str">
+        <v>dungtoan1</v>
+      </c>
+      <c r="C24" t="str">
+        <v>dung</v>
+      </c>
+      <c r="D24" t="str" xml:space="preserve">
+        <v xml:space="preserve">NguyenNguyenNguyenNguyenNguyenNguyenNguyenNguyenNguyenNguyenNguyenNguyenNguyenNguyenNguyenNguyen
+</v>
+      </c>
+      <c r="E24" t="str">
+        <v>DUNG</v>
+      </c>
+      <c r="F24" t="str">
+        <v>dung@gmail.com</v>
+      </c>
+      <c r="J24" t="str">
+        <v>Thông tin tài khoản đã được cập nhật.</v>
+      </c>
+    </row>
+    <row r="25" xml:space="preserve">
+      <c r="A25" t="str">
+        <v>dung@gmail.com</v>
+      </c>
+      <c r="B25" t="str">
+        <v>dungtoan1</v>
+      </c>
+      <c r="C25" t="str">
+        <v>dung</v>
+      </c>
+      <c r="D25" t="str">
+        <v>nguyen</v>
+      </c>
+      <c r="E25" t="str">
+        <v>DUNG</v>
+      </c>
+      <c r="F25" t="str">
+        <v>dung@gmail.com</v>
+      </c>
+      <c r="H25" t="str" xml:space="preserve">
+        <v xml:space="preserve">DungAbc@1234567890Abc@1234567890Abc@1234567890Abc@1234567890Abc@1234567890Abc@1234567890
+</v>
+      </c>
+      <c r="I25" t="str" xml:space="preserve">
+        <v xml:space="preserve">DungAbc@1234567890Abc@1234567890Abc@1234567890Abc@1234567890Abc@1234567890Abc@1234567890
+</v>
+      </c>
+      <c r="J25" t="str">
+        <v>Thông tin tài khoản đã được cập nhật.</v>
+      </c>
+    </row>
+    <row r="26" xml:space="preserve">
+      <c r="A26" t="str">
+        <v>dung@gmail.com</v>
+      </c>
+      <c r="B26" t="str" xml:space="preserve">
+        <v xml:space="preserve">DungAbc@1234567890Abc@1234567890Abc@1234567890Abc@1234567890Abc@1234567890Abc@1234567890
+</v>
+      </c>
+      <c r="C26" t="str">
+        <v>doi_lai_mk_de_dnhap</v>
+      </c>
+      <c r="D26" t="str">
+        <v>nguyen</v>
+      </c>
+      <c r="E26" t="str">
+        <v>DUNG</v>
+      </c>
+      <c r="F26" t="str">
+        <v>dung@gmail.com</v>
+      </c>
+      <c r="G26" t="str">
+        <v>dungtoan1</v>
+      </c>
+      <c r="J26" t="str">
+        <v>Thông tin tài khoản đã được cập nhật.</v>
+      </c>
+    </row>
+    <row r="27" xml:space="preserve">
+      <c r="A27" t="str">
+        <v>dung@gmail.com</v>
+      </c>
+      <c r="B27" t="str">
+        <v>dungtoan1</v>
+      </c>
+      <c r="C27" t="str">
+        <v>dung</v>
+      </c>
+      <c r="D27" t="str">
+        <v>nguyen</v>
+      </c>
+      <c r="E27" t="str">
+        <v>DUNG</v>
+      </c>
+      <c r="F27" t="str" xml:space="preserve">
+        <v xml:space="preserve">aaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaabbbbbbbbbbbbbbbbbbbbbbbbbbbbbbbbbbbbbbbbbbbbbbbbbbbbbbbbbbbbbbbcccccccccccccccccccccccccccccccccccccccccccccccccccccccccccccccdddddddddddddddddddddddddddddddddddddddddddddddddddddddd@eeeeeefffffffffffffffffffffffffffffffffffffffffffffffffffffffffff.com
+</v>
+      </c>
+      <c r="J27" t="str">
+        <v>Please enter an email address.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J22"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J27"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1741,7 +1887,7 @@
         <v>không</v>
       </c>
       <c r="I4" t="str">
-        <v>Mục Thị trấn / Thành phố là mục bắt buộc .</v>
+        <v>Mục Thị trấn / Thành phố là mục bắt buộc.</v>
       </c>
     </row>
     <row r="5">
@@ -1799,7 +1945,7 @@
         <v>không</v>
       </c>
       <c r="I6" t="str">
-        <v>Mục Địa chỉ email là mục bắt buộc .</v>
+        <v>Mục Địa chỉ email là mục bắt buộc.</v>
       </c>
     </row>
     <row r="7">
@@ -1857,7 +2003,7 @@
         <v>không</v>
       </c>
       <c r="I8" t="str" xml:space="preserve">
-        <v xml:space="preserve">Mục Tên là mục bắt buộc._x000d_
+        <v xml:space="preserve">Mục Tên là mục bắt buộc._x000d__x000d__x000d__x000d_
 Mục Địa chỉ là mục bắt buộc.</v>
       </c>
     </row>
@@ -1887,7 +2033,7 @@
         <v/>
       </c>
       <c r="I9" t="str">
-        <v>Mục Địa chỉ email không phải là địa chỉ email hợp lệ.</v>
+        <v>Mục Địa chỉ email không phải là địa chỉ email hợp lệ.</v>
       </c>
     </row>
     <row r="10">
@@ -1916,7 +2062,7 @@
         <v/>
       </c>
       <c r="I10" t="str">
-        <v>Mục Địa chỉ email không phải là địa chỉ email hợp lệ.</v>
+        <v>Mục Địa chỉ email không phải là địa chỉ email hợp lê.</v>
       </c>
     </row>
     <row r="11">

</xml_diff>